<commit_message>
Correção de bugs e continuação do projeto em casa
</commit_message>
<xml_diff>
--- a/Base_Mestra_FDE.xlsx
+++ b/Base_Mestra_FDE.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base_Mestra_FDE" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Base_Mestra_FDE" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resumo" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,8 +42,11 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -63,6 +66,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFACD"/>
       </patternFill>
     </fill>
   </fills>
@@ -92,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -110,6 +118,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -475,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3161"/>
+  <dimension ref="A1:C3190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -54001,6 +54015,499 @@
       <c r="C3161" s="4" t="inlineStr">
         <is>
           <t>MV</t>
+        </is>
+      </c>
+    </row>
+    <row r="3162">
+      <c r="A3162" s="7" t="inlineStr">
+        <is>
+          <t>03.00.000</t>
+        </is>
+      </c>
+      <c r="B3162" s="8" t="inlineStr">
+        <is>
+          <t>ESTRUTURA</t>
+        </is>
+      </c>
+      <c r="C3162" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3163">
+      <c r="A3163" s="7" t="inlineStr">
+        <is>
+          <t>03.02.000</t>
+        </is>
+      </c>
+      <c r="B3163" s="8" t="inlineStr">
+        <is>
+          <t>ESTRUTURA - SUPER ESTRUTURA</t>
+        </is>
+      </c>
+      <c r="C3163" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3164">
+      <c r="A3164" s="7" t="inlineStr">
+        <is>
+          <t>03.04.000</t>
+        </is>
+      </c>
+      <c r="B3164" s="8" t="inlineStr">
+        <is>
+          <t>ESTRUTURA - ESTRUTURA METÁLICA</t>
+        </is>
+      </c>
+      <c r="C3164" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3165">
+      <c r="A3165" s="7" t="inlineStr">
+        <is>
+          <t>06.85.000</t>
+        </is>
+      </c>
+      <c r="B3165" s="8" t="inlineStr">
+        <is>
+          <t>ESQ. METÁLICAS - RETIRADAS DE FERRAGENS</t>
+        </is>
+      </c>
+      <c r="C3165" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3166">
+      <c r="A3166" s="7" t="inlineStr">
+        <is>
+          <t>07.00.000</t>
+        </is>
+      </c>
+      <c r="B3166" s="8" t="inlineStr">
+        <is>
+          <t>COBERTURA</t>
+        </is>
+      </c>
+      <c r="C3166" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3167">
+      <c r="A3167" s="7" t="inlineStr">
+        <is>
+          <t>07.02.000</t>
+        </is>
+      </c>
+      <c r="B3167" s="8" t="inlineStr">
+        <is>
+          <t>COBERTURA - ESTRUTURA METÁLICA</t>
+        </is>
+      </c>
+      <c r="C3167" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3168">
+      <c r="A3168" s="7" t="inlineStr">
+        <is>
+          <t>07.03.000</t>
+        </is>
+      </c>
+      <c r="B3168" s="8" t="inlineStr">
+        <is>
+          <t>COBERTURA - TELHAS</t>
+        </is>
+      </c>
+      <c r="C3168" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3169">
+      <c r="A3169" s="7" t="inlineStr">
+        <is>
+          <t>07.04.000</t>
+        </is>
+      </c>
+      <c r="B3169" s="8" t="inlineStr">
+        <is>
+          <t>COBERTURA - CUMEEIRAS E RUFOS</t>
+        </is>
+      </c>
+      <c r="C3169" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3170">
+      <c r="A3170" s="7" t="inlineStr">
+        <is>
+          <t>07.05.000</t>
+        </is>
+      </c>
+      <c r="B3170" s="8" t="inlineStr">
+        <is>
+          <t>COBERTURA - FECHAMENTOS E VEDAÇÕES</t>
+        </is>
+      </c>
+      <c r="C3170" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3171">
+      <c r="A3171" s="7" t="inlineStr">
+        <is>
+          <t>08.00.000</t>
+        </is>
+      </c>
+      <c r="B3171" s="8" t="inlineStr">
+        <is>
+          <t>INST. HIDRÁULICAS E SANITÁRIAS</t>
+        </is>
+      </c>
+      <c r="C3171" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3172">
+      <c r="A3172" s="7" t="inlineStr">
+        <is>
+          <t>08.05.000</t>
+        </is>
+      </c>
+      <c r="B3172" s="8" t="inlineStr">
+        <is>
+          <t>INST. HIDRÁULICAS - TUBOS DE COBRE</t>
+        </is>
+      </c>
+      <c r="C3172" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3173">
+      <c r="A3173" s="7" t="inlineStr">
+        <is>
+          <t>08.07.000</t>
+        </is>
+      </c>
+      <c r="B3173" s="8" t="inlineStr">
+        <is>
+          <t>INST. HIDRÁULICAS - ÁGUA FRIA</t>
+        </is>
+      </c>
+      <c r="C3173" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3174">
+      <c r="A3174" s="7" t="inlineStr">
+        <is>
+          <t>08.08.000</t>
+        </is>
+      </c>
+      <c r="B3174" s="8" t="inlineStr">
+        <is>
+          <t>INST. HIDRÁULICAS - ESGOTO</t>
+        </is>
+      </c>
+      <c r="C3174" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3175">
+      <c r="A3175" s="7" t="inlineStr">
+        <is>
+          <t>08.11.000</t>
+        </is>
+      </c>
+      <c r="B3175" s="8" t="inlineStr">
+        <is>
+          <t>INST. HIDRÁULICAS - ÁGUAS PLUVIAIS TUBULAÇÕES</t>
+        </is>
+      </c>
+      <c r="C3175" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3176">
+      <c r="A3176" s="7" t="inlineStr">
+        <is>
+          <t>08.12.000</t>
+        </is>
+      </c>
+      <c r="B3176" s="8" t="inlineStr">
+        <is>
+          <t>INST. HIDRÁULICAS - ÁGUAS PLUVIAIS CALHAS</t>
+        </is>
+      </c>
+      <c r="C3176" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3177">
+      <c r="A3177" s="7" t="inlineStr">
+        <is>
+          <t>08.13.000</t>
+        </is>
+      </c>
+      <c r="B3177" s="8" t="inlineStr">
+        <is>
+          <t>INST. HIDRÁULICAS - TUBULAÇÕES GERAIS</t>
+        </is>
+      </c>
+      <c r="C3177" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3178">
+      <c r="A3178" s="7" t="inlineStr">
+        <is>
+          <t>08.84.000</t>
+        </is>
+      </c>
+      <c r="B3178" s="8" t="inlineStr">
+        <is>
+          <t>INST. HIDRÁULICAS - PEÇAS DE REPOSIÇÃO SANITÁRIA</t>
+        </is>
+      </c>
+      <c r="C3178" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3179">
+      <c r="A3179" s="7" t="inlineStr">
+        <is>
+          <t>09.00.000</t>
+        </is>
+      </c>
+      <c r="B3179" s="8" t="inlineStr">
+        <is>
+          <t>INST. ELÉTRICAS E LÓGICA</t>
+        </is>
+      </c>
+      <c r="C3179" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3180">
+      <c r="A3180" s="7" t="inlineStr">
+        <is>
+          <t>09.05.000</t>
+        </is>
+      </c>
+      <c r="B3180" s="8" t="inlineStr">
+        <is>
+          <t>INST. ELÉTRICAS - ELETRODUTOS</t>
+        </is>
+      </c>
+      <c r="C3180" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3181">
+      <c r="A3181" s="7" t="inlineStr">
+        <is>
+          <t>09.07.000</t>
+        </is>
+      </c>
+      <c r="B3181" s="8" t="inlineStr">
+        <is>
+          <t>INST. ELÉTRICAS - FIOS E CABOS</t>
+        </is>
+      </c>
+      <c r="C3181" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3182">
+      <c r="A3182" s="7" t="inlineStr">
+        <is>
+          <t>09.08.000</t>
+        </is>
+      </c>
+      <c r="B3182" s="8" t="inlineStr">
+        <is>
+          <t>INST. ELÉTRICAS - PONTOS ELÉTRICOS</t>
+        </is>
+      </c>
+      <c r="C3182" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3183">
+      <c r="A3183" s="7" t="inlineStr">
+        <is>
+          <t>09.09.000</t>
+        </is>
+      </c>
+      <c r="B3183" s="8" t="inlineStr">
+        <is>
+          <t>INST. ELÉTRICAS - ILUMINAÇÃO</t>
+        </is>
+      </c>
+      <c r="C3183" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3184">
+      <c r="A3184" s="7" t="inlineStr">
+        <is>
+          <t>09.13.000</t>
+        </is>
+      </c>
+      <c r="B3184" s="8" t="inlineStr">
+        <is>
+          <t>INST. ELÉTRICAS - SPDA/ATERRAMENTO</t>
+        </is>
+      </c>
+      <c r="C3184" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3185">
+      <c r="A3185" s="7" t="inlineStr">
+        <is>
+          <t>09.82.000</t>
+        </is>
+      </c>
+      <c r="B3185" s="8" t="inlineStr">
+        <is>
+          <t>INST. ELÉTRICAS - POSTES E SUPORTES</t>
+        </is>
+      </c>
+      <c r="C3185" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3186">
+      <c r="A3186" s="7" t="inlineStr">
+        <is>
+          <t>09.84.000</t>
+        </is>
+      </c>
+      <c r="B3186" s="8" t="inlineStr">
+        <is>
+          <t>INST. ELÉTRICAS - INTERRUPTORES E TOMADAS</t>
+        </is>
+      </c>
+      <c r="C3186" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3187">
+      <c r="A3187" s="7" t="inlineStr">
+        <is>
+          <t>09.85.000</t>
+        </is>
+      </c>
+      <c r="B3187" s="8" t="inlineStr">
+        <is>
+          <t>INST. ELÉTRICAS - INFRAESTRUTURA LÓGICA</t>
+        </is>
+      </c>
+      <c r="C3187" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3188">
+      <c r="A3188" s="7" t="inlineStr">
+        <is>
+          <t>15.00.000</t>
+        </is>
+      </c>
+      <c r="B3188" s="8" t="inlineStr">
+        <is>
+          <t>PINTURAS</t>
+        </is>
+      </c>
+      <c r="C3188" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3189">
+      <c r="A3189" s="7" t="inlineStr">
+        <is>
+          <t>15.01.000</t>
+        </is>
+      </c>
+      <c r="B3189" s="8" t="inlineStr">
+        <is>
+          <t>PINTURAS - ESTRUTURA METÁLICA</t>
+        </is>
+      </c>
+      <c r="C3189" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3190">
+      <c r="A3190" s="7" t="inlineStr">
+        <is>
+          <t>15.03.000</t>
+        </is>
+      </c>
+      <c r="B3190" s="8" t="inlineStr">
+        <is>
+          <t>PINTURAS - ESQUADRIAS METÁLICAS</t>
+        </is>
+      </c>
+      <c r="C3190" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
         </is>
       </c>
     </row>

</xml_diff>